<commit_message>
Carrier-ready semantics + money held up: rescrubbed site copy, fresh sample report/dashboard
</commit_message>
<xml_diff>
--- a/sample-report.xlsx
+++ b/sample-report.xlsx
@@ -16,8 +16,8 @@
     <sheet name="Processing Log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$B$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Loads'!$A$1:$S$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Loads'!$A$1:$W$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exceptions'!$A$1:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Documents'!$A$1:$AC$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Line Items'!$A$1:$H$30</definedName>
@@ -56,7 +56,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +71,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -91,13 +96,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -466,14 +479,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -487,14 +500,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What to invoice now, and what's blocking the rest. Detail tabs follow.</t>
+          <t>Carrier payables ready for review, and what's blocking the rest. Amounts are contracted carrier rates, not customer invoice amounts. Detail tabs follow.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>INVOICE THESE NOW — 5 load(s) billing-ready</t>
+          <t>CARRIER PAYABLES READY — 5 load(s)</t>
         </is>
       </c>
     </row>
@@ -506,7 +519,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Carrier</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -521,7 +534,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Carrier amount</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -530,354 +543,389 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1001</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Capital City Grocers</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Red Mesa Trucking LLC</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Dallas, TX → Memphis, TN</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>$3,388.23</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="5" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1002</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Riverbend Manufacturing</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Sierra Freight Lines LLC</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Houston, TX → Atlanta, GA</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>$2,409.43</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="5" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1003</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Capital City Grocers</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Bluebonnet Express LLC</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Mobile, AL → Jackson, MS</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>$2,266.89</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="5" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Lone Star Retail DC</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Red Mesa Trucking LLC</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>San Antonio, TX → Little Rock, AR</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="5" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1011</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Delta Foods Warehouse</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Red Mesa Trucking LLC</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Houston, TX → Atlanta, GA</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>$2,276.57</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="5" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>BLOCKED — 6 load(s) need attention</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>CUSTOMER INVOICING</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Customer invoice readiness is not determined from these documents. Carrier documents do not show the customer sell rate or the bill-to party. Do not invoice a customer based on the carrier amounts above.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>BLOCKED — 6 load(s) need attention — $23,826.51 in carrier payables held up</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Load</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Carrier</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>What's blocking</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1004</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Lone Star Retail DC</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Red Mesa Trucking LLC</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Baton Rouge, LA → Nashville, TN</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Invoice totals are inconsistent.; 2 high-severity exception(s) open.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Check invoice totals against the rate confirmation</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Carrier invoice totals are inconsistent with the rate.; 2 high-severity exception(s) open. Missing: Bill of Lading.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Confirm the rate with the broker</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1005</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Sunbelt Home Centers</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Red Mesa Trucking LLC</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Baton Rouge, LA → Nashville, TN</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>2 high-severity exception(s) open.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Review the Exceptions tab for details</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>LD-2026-1006</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Lone Star Retail DC</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Coyote Canyon Carriers</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>San Antonio, TX → Little Rock, AR</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>No signed proof of delivery.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>No signed proof of delivery. Missing: Bill of Lading, Proof of Delivery, Commercial Invoice.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Chase the signed POD from the carrier/driver</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>LD-2026-1007</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Delta Pine Hauling Co</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Mobile, AL → Jackson, MS</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>No signed proof of delivery.; 1 high-severity exception(s) open. Missing: Bill of Lading.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Chase the signed POD from the carrier/driver</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>LD-2026-1009</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Sierra Freight Lines LLC</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio, TX → Little Rock, AR</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>1 high-severity exception(s) open.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Review the Exceptions tab for details</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>LD-2026-1007</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Riverbend Manufacturing</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Mobile, AL → Jackson, MS</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>No signed proof of delivery.; 1 high-severity exception(s) open.</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>LD-2026-1012</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Delta Pine Hauling Co</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>New Orleans, LA → Birmingham, AL</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>1 high-severity exception(s) open.</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Review the Exceptions tab for details</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>LD-2026-1009</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Lone Star Retail DC</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>San Antonio, TX → Little Rock, AR</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>1 high-severity exception(s) open.</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Review the Exceptions tab for details</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>LD-2026-1012</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Capital City Grocers</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>New Orleans, LA → Birmingham, AL</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>1 high-severity exception(s) open.</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Review the Exceptions tab for details</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
@@ -891,20 +939,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -943,7 +991,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Billing-ready loads</t>
+          <t>Carrier-ready loads (payable)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -953,55 +1001,89 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total exceptions</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>13</v>
+          <t>Carrier payables held up by incomplete paperwork</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$23,826.51</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High-severity exceptions</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>7</v>
+          <t>Customer receivables held up</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Not determinable — carrier documents do not show customer sell rates</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Missing POD signatures</t>
+          <t>Total exceptions</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Flagged for human review</t>
+          <t>High-severity exceptions</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Loads with no POD document</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PODs present but unsigned</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Flagged for human review</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Average extraction confidence</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B13" t="n">
         <v>0.973</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1012,7 +1094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:W12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1034,100 +1116,124 @@
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="48" customWidth="1" min="18" max="18"/>
     <col width="48" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="48" customWidth="1" min="22" max="22"/>
+    <col width="48" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>load_number</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>shipper</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>consignee</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>carrier</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>broker</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>origin</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>destination</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>ship_date</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>delivery_date</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>commodity</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>weight_lbs</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>pieces</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>rc_total</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>invoice_total</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>pod_signed</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="P1" s="8" t="inlineStr">
         <is>
           <t>doc_count</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
-        <is>
-          <t>billing_ready</t>
-        </is>
-      </c>
-      <c r="R1" s="6" t="inlineStr">
-        <is>
-          <t>billing_blockers</t>
-        </is>
-      </c>
-      <c r="S1" s="6" t="inlineStr">
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>carrier_ready</t>
+        </is>
+      </c>
+      <c r="R1" s="8" t="inlineStr">
+        <is>
+          <t>carrier_blockers</t>
+        </is>
+      </c>
+      <c r="S1" s="8" t="inlineStr">
+        <is>
+          <t>missing_documents</t>
+        </is>
+      </c>
+      <c r="T1" s="8" t="inlineStr">
+        <is>
+          <t>held_up_carrier_amount</t>
+        </is>
+      </c>
+      <c r="U1" s="8" t="inlineStr">
+        <is>
+          <t>customer_ready</t>
+        </is>
+      </c>
+      <c r="V1" s="8" t="inlineStr">
+        <is>
+          <t>customer_blockers</t>
+        </is>
+      </c>
+      <c r="W1" s="8" t="inlineStr">
         <is>
           <t>source_files</t>
         </is>
@@ -1211,6 +1317,21 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
           <t>bil-L01-02.pdf, com-L01-04.pdf, pro-L01-03.pdf, rat-L01-01.pdf</t>
         </is>
       </c>
@@ -1293,6 +1414,21 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
           <t>bil-L02-06.pdf, com-L02-08.xlsx, pro-L02-07.xlsx, rat-L02-05.xlsx</t>
         </is>
       </c>
@@ -1375,6 +1511,21 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
           <t>bil-L03-10.csv, com-L03-12.csv, pro-L03-11.pdf, rat-L03-09.csv</t>
         </is>
       </c>
@@ -1457,10 +1608,28 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Invoice totals are inconsistent.; 2 high-severity exception(s) open.</t>
+          <t>Carrier invoice totals are inconsistent with the rate.; 2 high-severity exception(s) open.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
+        <is>
+          <t>Bill of Lading</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>3607.91</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
         <is>
           <t>com-L04-15.pdf, pro-L04-14.pdf, rat-L04-13.pdf</t>
         </is>
@@ -1549,6 +1718,24 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>3241.95</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
           <t>bil-L05-17.pdf, com-L05-19.pdf, pro-L05-18.pdf, rat-L05-16.pdf</t>
         </is>
       </c>
@@ -1633,6 +1820,24 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
+          <t>Bill of Lading, Proof of Delivery, Commercial Invoice</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>4460.76</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
           <t>rat-L06-20.pdf</t>
         </is>
       </c>
@@ -1720,6 +1925,24 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
+          <t>Bill of Lading</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>4270.94</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
           <t>com-L07-22.pdf, com-L07-24.pdf, pro-L07-23.pdf, rat-L07-21.pdf</t>
         </is>
       </c>
@@ -1791,6 +2014,21 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
+          <t>Rate Confirmation, Commercial Invoice</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
           <t>bil-L08-25.pdf, pro-L08-26.pdf</t>
         </is>
       </c>
@@ -1878,6 +2116,24 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>4753.52</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
           <t>bil-L09-28.pdf, com-L09-30.pdf, pro-L09-29.pdf, rat-L09-27.pdf</t>
         </is>
       </c>
@@ -1960,6 +2216,21 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
           <t>bil-L11-33.pdf, com-L11-35.pdf, pro-L11-34.pdf, rat-L11-32.pdf</t>
         </is>
       </c>
@@ -2047,12 +2318,30 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>3491.43</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Customer sell rate not established — carrier documents do not show the customer invoice amount or the bill-to party.</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
           <t>bil-L12-37.pdf, com-L12-39.pdf, pro-L12-38.pdf, rat-L12-36.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S12"/>
+  <autoFilter ref="A1:W12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2078,47 +2367,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>exception_id</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>check</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>doc_id</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>doc_type</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>load_number</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>message</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>page</t>
         </is>
@@ -2772,147 +3061,147 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>doc_id</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>doc_type</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>page</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>load_number</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>bol_number</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>invoice_number</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>po_number</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>ship_date</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>delivery_date</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>invoice_date</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>shipper</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>consignee</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>carrier</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>broker</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="P1" s="8" t="inlineStr">
         <is>
           <t>origin</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
+      <c r="Q1" s="8" t="inlineStr">
         <is>
           <t>destination</t>
         </is>
       </c>
-      <c r="R1" s="6" t="inlineStr">
+      <c r="R1" s="8" t="inlineStr">
         <is>
           <t>commodity</t>
         </is>
       </c>
-      <c r="S1" s="6" t="inlineStr">
+      <c r="S1" s="8" t="inlineStr">
         <is>
           <t>weight_lbs</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="T1" s="8" t="inlineStr">
         <is>
           <t>pieces</t>
         </is>
       </c>
-      <c r="U1" s="6" t="inlineStr">
+      <c r="U1" s="8" t="inlineStr">
         <is>
           <t>linehaul</t>
         </is>
       </c>
-      <c r="V1" s="6" t="inlineStr">
+      <c r="V1" s="8" t="inlineStr">
         <is>
           <t>fuel_surcharge</t>
         </is>
       </c>
-      <c r="W1" s="6" t="inlineStr">
+      <c r="W1" s="8" t="inlineStr">
         <is>
           <t>accessorials</t>
         </is>
       </c>
-      <c r="X1" s="6" t="inlineStr">
+      <c r="X1" s="8" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="Y1" s="6" t="inlineStr">
+      <c r="Y1" s="8" t="inlineStr">
         <is>
           <t>pod_signed</t>
         </is>
       </c>
-      <c r="Z1" s="6" t="inlineStr">
+      <c r="Z1" s="8" t="inlineStr">
         <is>
           <t>received_by</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
+      <c r="AA1" s="8" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="AB1" s="6" t="inlineStr">
+      <c r="AB1" s="8" t="inlineStr">
         <is>
           <t>needs_review</t>
         </is>
       </c>
-      <c r="AC1" s="6" t="inlineStr">
+      <c r="AC1" s="8" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -3258,7 +3547,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3425,7 +3714,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3886,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3965,7 +4254,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4346,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4149,7 +4438,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4530,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4622,7 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4893,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4816,7 +5105,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4869,7 +5158,7 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4917,7 +5206,7 @@
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5023,7 +5312,7 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5418,7 @@
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5541,7 +5830,7 @@
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5933,7 @@
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5850,7 +6139,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5953,7 +6242,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6154,7 +6443,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6232,42 +6521,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>doc_id</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>doc_type</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>load_number</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>commodity</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>weight_lbs</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>pieces</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>page</t>
         </is>
@@ -7326,22 +7615,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>file</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>docs</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>ts</t>
         </is>
@@ -7363,7 +7652,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7672,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7403,7 +7692,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7423,7 +7712,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7443,7 +7732,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7752,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7483,7 +7772,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7503,7 +7792,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7812,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7543,7 +7832,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7563,7 +7852,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7583,7 +7872,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7603,7 +7892,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7623,7 +7912,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7643,7 +7932,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7663,7 +7952,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7683,7 +7972,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7992,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7723,7 +8012,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7743,7 +8032,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7763,7 +8052,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7783,7 +8072,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7803,7 +8092,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7823,7 +8112,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7843,7 +8132,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7863,7 +8152,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7883,7 +8172,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7903,7 +8192,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7923,7 +8212,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7943,7 +8232,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7963,7 +8252,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -7983,7 +8272,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8003,7 +8292,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:52+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8312,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:53+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8043,7 +8332,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:53+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8063,7 +8352,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:53+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8083,7 +8372,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:53+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8103,7 +8392,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:53+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8123,7 +8412,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:53+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>
@@ -8143,7 +8432,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-10-08T06:58:53+00:00</t>
+          <t>2026-10-11T05:13:17+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate samples with fixed readiness logic
- LD-2026-1008 now NOT READY (was incorrectly CARRIER READY with missing docs)
- LD-2026-1011 now NOT READY (was incorrectly CARRIER READY with missing carrier field)
- 3 carrier-ready loads (was 5) with stricter validation
</commit_message>
<xml_diff>
--- a/sample-report.xlsx
+++ b/sample-report.xlsx
@@ -507,7 +507,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CARRIER PAYABLES READY — 5 load(s)</t>
+          <t>CARRIER PAYABLES READY — 3 load(s)</t>
         </is>
       </c>
     </row>
@@ -633,196 +633,190 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>LD-2026-1008</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>CUSTOMER INVOICING</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Customer invoice readiness is not determined from these documents. Carrier documents do not show the customer sell rate or the bill-to party. Do not invoice a customer based on the carrier amounts above.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>BLOCKED — 8 load(s) need attention — $26,103.08 in carrier payables held up</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Carrier</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>What's blocking</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Next step</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>LD-2026-1004</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Red Mesa Trucking LLC</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>San Antonio, TX → Little Rock, AR</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>LD-2026-1011</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Baton Rouge, LA → Nashville, TN</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Missing required documents: Bill of Lading.; Carrier invoice totals are inconsistent with the rate.; 2 blocking exception(s) open. Missing: Bill of Lading.</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Reconcile the invoice against the agreed rate confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>LD-2026-1005</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Red Mesa Trucking LLC</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Houston, TX → Atlanta, GA</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>$2,276.57</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>CUSTOMER INVOICING</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Customer invoice readiness is not determined from these documents. Carrier documents do not show the customer sell rate or the bill-to party. Do not invoice a customer based on the carrier amounts above.</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>BLOCKED — 6 load(s) need attention — $23,826.51 in carrier payables held up</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Carrier</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>What's blocking</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Next step</t>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Baton Rouge, LA → Nashville, TN</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>2 blocking exception(s) open.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Review the Exceptions tab for details</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>LD-2026-1004</t>
+          <t>LD-2026-1006</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Red Mesa Trucking LLC</t>
+          <t>Coyote Canyon Carriers</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Baton Rouge, LA → Nashville, TN</t>
+          <t>San Antonio, TX → Little Rock, AR</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Carrier invoice totals are inconsistent with the rate.; 2 high-severity exception(s) open. Missing: Bill of Lading.</t>
+          <t>Missing required documents: Bill of Lading, Commercial Invoice, Proof of Delivery. Missing: Bill of Lading, Proof of Delivery, Commercial Invoice.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Confirm the rate with the broker</t>
+          <t>Chase the signed POD from the carrier/driver</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>LD-2026-1005</t>
+          <t>LD-2026-1007</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Red Mesa Trucking LLC</t>
+          <t>Delta Pine Hauling Co</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Baton Rouge, LA → Nashville, TN</t>
+          <t>Mobile, AL → Jackson, MS</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>2 high-severity exception(s) open.</t>
+          <t>Missing required documents: Bill of Lading.; No signed proof of delivery.; 3 blocking exception(s) open. Missing: Bill of Lading.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Review the Exceptions tab for details</t>
+          <t>Request the signed delivery POD from the carrier/driver</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>LD-2026-1006</t>
+          <t>LD-2026-1008</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Coyote Canyon Carriers</t>
+          <t>Red Mesa Trucking LLC</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -832,61 +826,61 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>No signed proof of delivery. Missing: Bill of Lading, Proof of Delivery, Commercial Invoice.</t>
+          <t>Missing required documents: Commercial Invoice, Rate Confirmation.; 1 blocking exception(s) open. Missing: Rate Confirmation, Commercial Invoice.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Chase the signed POD from the carrier/driver</t>
+          <t>Confirm the rate with the broker</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>LD-2026-1007</t>
+          <t>LD-2026-1009</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Delta Pine Hauling Co</t>
+          <t>Sierra Freight Lines LLC</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Mobile, AL → Jackson, MS</t>
+          <t>San Antonio, TX → Little Rock, AR</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>No signed proof of delivery.; 1 high-severity exception(s) open. Missing: Bill of Lading.</t>
+          <t>1 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Chase the signed POD from the carrier/driver</t>
+          <t>Review the Exceptions tab for details</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>LD-2026-1009</t>
+          <t>LD-2026-1011</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Sierra Freight Lines LLC</t>
+          <t>Red Mesa Trucking LLC</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>San Antonio, TX → Little Rock, AR</t>
+          <t>Houston, TX → Atlanta, GA</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>1 high-severity exception(s) open.</t>
+          <t>1 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -913,7 +907,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>1 high-severity exception(s) open.</t>
+          <t>1 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -924,10 +918,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -995,7 +989,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -1006,7 +1000,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$23,826.51</t>
+          <t>$26,103.08</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1063,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
@@ -1608,7 +1602,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Carrier invoice totals are inconsistent with the rate.; 2 high-severity exception(s) open.</t>
+          <t>Missing required documents: Bill of Lading.; Carrier invoice totals are inconsistent with the rate.; 2 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -1713,7 +1707,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2 high-severity exception(s) open.</t>
+          <t>2 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1815,7 +1809,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>No signed proof of delivery.</t>
+          <t>Missing required documents: Bill of Lading, Commercial Invoice, Proof of Delivery.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1920,7 +1914,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>No signed proof of delivery.; 1 high-severity exception(s) open.</t>
+          <t>Missing required documents: Bill of Lading.; No signed proof of delivery.; 3 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2009,7 +2003,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Missing required documents: Commercial Invoice, Rate Confirmation.; 1 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -2111,7 +2110,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1 high-severity exception(s) open.</t>
+          <t>1 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -2211,13 +2210,21 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
+      </c>
+      <c r="T11" t="n">
+        <v>2276.57</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
@@ -2313,7 +2320,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1 high-severity exception(s) open.</t>
+          <t>1 blocking exception(s) open.</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -3628,7 +3635,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4716,7 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6340,7 +6347,7 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -7652,7 +7659,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7672,7 +7679,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7692,7 +7699,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7712,7 +7719,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7732,7 +7739,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7759,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7779,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:38+00:00</t>
         </is>
       </c>
     </row>
@@ -7792,7 +7799,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7819,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7832,7 +7839,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7852,7 +7859,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7879,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7892,7 +7899,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7912,7 +7919,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7932,7 +7939,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7952,7 +7959,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7972,7 +7979,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7999,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8012,7 +8019,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8032,7 +8039,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8052,7 +8059,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8072,7 +8079,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8099,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8112,7 +8119,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8132,7 +8139,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8152,7 +8159,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8172,7 +8179,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8192,7 +8199,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8212,7 +8219,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8232,7 +8239,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8252,7 +8259,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8279,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8292,7 +8299,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8312,7 +8319,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8332,7 +8339,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8352,7 +8359,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8372,7 +8379,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8399,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8412,7 +8419,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8439,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-10-11T05:13:17+00:00</t>
+          <t>2026-10-12T06:08:39+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>